<commit_message>
[ENH] Bug solving and added automatic graph generation of staircase tests at the end
</commit_message>
<xml_diff>
--- a/src/CEACO_image_selection.xlsx
+++ b/src/CEACO_image_selection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D7B3ED-ADB3-436F-9DC4-AC15CBF59013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE03CF4B-A0D1-413D-8448-14F6B314CDB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="33">
   <si>
     <t>arousal</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>..\..\2.DATASETS\CEACO\EM0701_0800\EM0792.jpg</t>
-  </si>
-  <si>
-    <t>..\..\2.DATASETS\CEACO\EM1101_1202\EM1190.jpg</t>
   </si>
   <si>
     <t>..\..\2.DATASETS\CEACO\EM0101_0200\EM0188.jpg</t>
@@ -444,7 +441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
@@ -669,7 +666,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B21" t="s">
         <v>4</v>
@@ -708,7 +705,7 @@
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
@@ -719,7 +716,7 @@
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
@@ -741,7 +738,7 @@
         <v>4</v>
       </c>
       <c r="C27" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.45">
@@ -752,7 +749,7 @@
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.45">
@@ -763,29 +760,7 @@
         <v>4</v>
       </c>
       <c r="C29" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A30" t="s">
-        <v>2</v>
-      </c>
-      <c r="B30" t="s">
-        <v>4</v>
-      </c>
-      <c r="C30" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
-        <v>2</v>
-      </c>
-      <c r="B31" t="s">
-        <v>4</v>
-      </c>
-      <c r="C31" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>